<commit_message>
herramientas-mx: validacion documental con fuente del fabricante y re-acomodo (sesion nocturna 1, #330)
- Cotas oficiales de cajon: 8444 = 58 mm (no 61), 8447 = 63+63+127, 414 x 318.
- 8420 sin barra para candado: M18 y baterias pasan a cajon con barra.
- 91 piezas con nivel por medida; 42 cambian con fuente documental.
- Estrategia de acomodo 'fijo' y comparacion de bases.
- Precios Home Depot MX con fecha e IVA; total normalizado sin IVA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TeXFoDoFpVre8AKoL589gf
</commit_message>
<xml_diff>
--- a/docs/herramientas-mx/asignacion_y_compra.xlsx
+++ b/docs/herramientas-mx/asignacion_y_compra.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Fabricacion" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Asignacion_por_rol" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Reuso_inventario" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Cambios_sesion_nocturna" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -38,7 +39,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -48,6 +49,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00B71C1C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B5E20"/>
       </patternFill>
     </fill>
   </fills>
@@ -63,9 +69,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -433,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -459,7 +468,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>159742.85</v>
+        <v>166422.1</v>
       </c>
     </row>
     <row r="3">
@@ -469,7 +478,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99079.78999999999</v>
+        <v>105759.04</v>
       </c>
     </row>
     <row r="4">
@@ -479,7 +488,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>112491.3</v>
+        <v>113195.3</v>
       </c>
     </row>
     <row r="5">
@@ -499,7 +508,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15445.2</v>
+        <v>16521.3</v>
       </c>
     </row>
     <row r="7">
@@ -509,7 +518,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>307755.45</v>
+        <v>316214.8</v>
       </c>
     </row>
     <row r="8">
@@ -519,28 +528,381 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>247092.39</v>
+        <v>255551.74</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Renglones de herramienta SIN precio (cotizar)</t>
+          <t>TOTAL con precio conocido, normalizado SIN IVA (tienda / 1.16)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9</v>
+        <v>300352.37</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>TOTAL normalizado con IVA (x 1.16)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>348408.75</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Renglones de herramienta SIN precio (cotizar)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Tipo de cambio usado</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>17.64 MXN/USD (Odoo, 2026-09-27)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>concepto</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>antes (d8f4483)</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>ahora</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>diferencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Herramienta a comprar (conservador, solo renglones con precio)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>159742.85</v>
+      </c>
+      <c r="C2" t="n">
+        <v>166422.1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>6679.25</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Herramienta a comprar si aparecen las compras de Odoo posteriores al listado</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>99079.78999999999</v>
+      </c>
+      <c r="C3" t="n">
+        <v>105759.04</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6679.25</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Contenedores, candados y cables</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>112491.3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>113195.3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>RFID (tags + lector)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>20076.1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>20076.1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Filamento PETG</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>15445.2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>16521.3</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1076.1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TOTAL con precio conocido (MXN, mezcla de precios sin IVA pagados y precios de tienda)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>307755.45</v>
+      </c>
+      <c r="C7" t="n">
+        <v>316214.8</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8459.35</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TOTAL si aparecen las compras de Odoo</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>247092.39</v>
+      </c>
+      <c r="C8" t="n">
+        <v>255551.74</v>
+      </c>
+      <c r="D8" t="n">
+        <v>8459.35</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TOTAL con precio conocido, normalizado SIN IVA (tienda / 1.16)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>300352.37</v>
+      </c>
+      <c r="D9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TOTAL normalizado con IVA (x 1.16)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>348408.75</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Renglones de herramienta SIN precio (cotizar)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>9</v>
+      </c>
+      <c r="C11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Tipo de cambio usado</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>17.64 MXN/USD (Odoo, 2026-09-27)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>17.64 MXN/USD (Odoo, 2026-09-27)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CONTENEDOR</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>necesidad antes</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>necesidad ahora</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>a comprar ahora</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>48-22-8420</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>6</v>
+      </c>
+      <c r="C15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D15" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>48-22-8442</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>48-22-8443</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" t="n">
+        <v>7</v>
+      </c>
+      <c r="D17" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>48-22-8444</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>15</v>
+      </c>
+      <c r="C18" t="n">
+        <v>8</v>
+      </c>
+      <c r="D18" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>48-22-8447</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>POR QUE CAMBIO</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Mezcla de cajas del acomodo nuevo (base 8420 + 8443 + 8444 con M18 bajo candado; soldadura 2 x 8447); 5 renglones antes sin precio ya lo tienen (pagina Home Depot MX leida, IVA incluido); 8443 a $3,799 de la pagina HD MX (antes $3,399 de fragmento); PETG sube por mas cajones con pieza.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>IVA</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>La hoja Resumen trae ahora el total normalizado SIN IVA (precio de tienda / 1.16) y con IVA. Lo pagado en Odoo ya viene sin IVA.</t>
         </is>
       </c>
     </row>
@@ -602,7 +964,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1 x 48-22-8420 + 2 x 48-22-8444</t>
+          <t>1 x 48-22-8443 + 1 x 48-22-8444 + 1 x 48-22-8420</t>
         </is>
       </c>
     </row>
@@ -642,7 +1004,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1 x 48-22-8442 + 1 x 48-22-8444</t>
+          <t>2 x 48-22-8447</t>
         </is>
       </c>
     </row>
@@ -682,7 +1044,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1 x 48-22-8420 + 1 x 48-22-8442 + 1 x 48-22-8444</t>
+          <t>1 x 48-22-8442 + 1 x 48-22-8444 + 1 x 48-22-8420</t>
         </is>
       </c>
     </row>
@@ -770,13 +1132,13 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>22997.15</v>
+        <v>24046.2</v>
       </c>
       <c r="D2" t="n">
-        <v>13184</v>
+        <v>13369</v>
       </c>
       <c r="E2" t="n">
-        <v>36181.15</v>
+        <v>37415.2</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -794,13 +1156,13 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>7364.81</v>
+        <v>7482.31</v>
       </c>
       <c r="D3" t="n">
         <v>3733</v>
       </c>
       <c r="E3" t="n">
-        <v>11097.81</v>
+        <v>11215.31</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -818,13 +1180,13 @@
         <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>7715.58</v>
+        <v>8315.08</v>
       </c>
       <c r="D4" t="n">
-        <v>7804</v>
+        <v>7236</v>
       </c>
       <c r="E4" t="n">
-        <v>15519.58</v>
+        <v>15551.08</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -845,10 +1207,10 @@
         <v>5965.14</v>
       </c>
       <c r="D5" t="n">
-        <v>3518</v>
+        <v>3918</v>
       </c>
       <c r="E5" t="n">
-        <v>9483.139999999999</v>
+        <v>9883.139999999999</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1553,14 +1915,20 @@
       <c r="H13" t="n">
         <v>2</v>
       </c>
+      <c r="I13" t="n">
+        <v>215</v>
+      </c>
+      <c r="J13" t="n">
+        <v>430</v>
+      </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>COTIZAR (sin precio en listado, Odoo ni buscador)</t>
+          <t>Home Depot MX 17016 sku 128377, pagina leida 2026-09-28, IVA incluido</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>sin precio</t>
+          <t>tienda</t>
         </is>
       </c>
     </row>
@@ -1739,14 +2107,20 @@
       <c r="H17" t="n">
         <v>1</v>
       </c>
+      <c r="I17" t="n">
+        <v>1199</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1199</v>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>COTIZAR</t>
+          <t>Home Depot MX HBCW10XLS sku 217405, pagina leida 2026-09-28, IVA incluido</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>sin precio</t>
+          <t>tienda</t>
         </is>
       </c>
     </row>
@@ -1783,7 +2157,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>COTIZAR (hoy son dados sueltos P7-P35)</t>
+          <t>COTIZAR (HD MX 2026-09-28 solo la matraca H38ROTORATMX $1,155 IVA incluido; los dados son sueltos P7-P35)</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1823,14 +2197,20 @@
       <c r="H19" t="n">
         <v>4</v>
       </c>
+      <c r="I19" t="n">
+        <v>1177</v>
+      </c>
+      <c r="J19" t="n">
+        <v>4708</v>
+      </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>COTIZAR</t>
+          <t>Home Depot MX suma de 3 paginas leidas 2026-09-28 (H3DEXT6MX $167 + 106545 $495 + H38BB10MX $515), IVA incluido</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>sin precio</t>
+          <t>tienda</t>
         </is>
       </c>
     </row>
@@ -2003,14 +2383,20 @@
       <c r="H23" t="n">
         <v>0</v>
       </c>
+      <c r="I23" t="n">
+        <v>145</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>COTIZAR</t>
+          <t>Home Depot MX MH-16 sku 462668, pagina leida 2026-09-28, IVA incluido</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>sin precio</t>
+          <t>tienda</t>
         </is>
       </c>
     </row>
@@ -2095,7 +2481,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>COTIZAR</t>
+          <t>COTIZAR (HD MX 2026-09-28 tiene 2 de 3: redonda $97 y triangular $61, IVA incluido; falta media cana)</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -2664,19 +3050,19 @@
         <v>5</v>
       </c>
       <c r="I37" t="n">
-        <v>1777.55</v>
+        <v>1799</v>
       </c>
       <c r="J37" t="n">
-        <v>8887.75</v>
+        <v>8995</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>buscador OASA Norte</t>
+          <t>Home Depot MX 48-59-1812 sku 129465, pagina leida 2026-09-28, IVA incluido</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>tienda</t>
         </is>
       </c>
     </row>
@@ -2903,14 +3289,20 @@
       <c r="H42" t="n">
         <v>1</v>
       </c>
+      <c r="I42" t="n">
+        <v>235</v>
+      </c>
+      <c r="J42" t="n">
+        <v>235</v>
+      </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>COTIZAR</t>
+          <t>Home Depot MX CE100821 sku 127734, pagina leida 2026-09-28, IVA incluido</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>sin precio</t>
+          <t>tienda</t>
         </is>
       </c>
     </row>
@@ -4245,7 +4637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4303,32 +4695,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>48-22-8420</t>
+          <t>48-22-8443</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E2" t="n">
-        <v>5599</v>
+        <v>3799</v>
       </c>
       <c r="F2" t="n">
-        <v>33594</v>
+        <v>26593</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>buscador HerramientaElectrica.mx</t>
+          <t>Home Depot MX sku 165831, pagina leida 2026-09-28, IVA incluido</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>tienda</t>
         </is>
       </c>
     </row>
@@ -4339,19 +4731,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E3" t="n">
         <v>3614</v>
       </c>
       <c r="F3" t="n">
-        <v>46982</v>
+        <v>25298</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -4367,126 +4759,158 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>48-22-8442</t>
+          <t>48-22-8420</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E4" t="n">
-        <v>3952</v>
+        <v>5599</v>
       </c>
       <c r="F4" t="n">
-        <v>19760</v>
+        <v>33594</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>buscador HerramientaElectrica.mx (agotado)</t>
+          <t>buscador HerramientaElectrica.mx</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>media</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>48-22-8443</t>
+          <t>48-22-8447</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>3399</v>
+        <v>3499</v>
       </c>
       <c r="F5" t="n">
-        <v>6798</v>
+        <v>10497</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>buscador Home Depot MX</t>
+          <t>Odoo P05566 (2026-02-04, sin IVA)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>pagado</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Candado de combinacion (1 por contenedor)</t>
+          <t>48-22-8442</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>119</v>
+        <v>3952</v>
       </c>
       <c r="F6" t="n">
-        <v>3332</v>
+        <v>11856</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>listado hoja Maleta Personal: Master 646DMX, Home Depot</t>
+          <t>buscador HerramientaElectrica.mx (agotado)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>pagado</t>
+          <t>alta</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Candado de combinacion (1 por contenedor)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>28</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>28</v>
+      </c>
+      <c r="E7" t="n">
+        <v>119</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3332</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>listado hoja Maleta Personal: Master 646DMX, Home Depot</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>pagado</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Cable de acero con candado para resguardo (1 por kit + 1 por modulo con 8420)</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B8" t="n">
         <v>6</v>
       </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
         <v>6</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E8" t="n">
         <v>337.55</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F8" t="n">
         <v>2025.3</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>buscador Amazon MX: cable 1.8 m con combinacion reajustable</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>baja</t>
         </is>
@@ -5222,13 +5646,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>24.4</v>
+        <v>26.1</v>
       </c>
       <c r="C2" t="n">
         <v>633</v>
       </c>
       <c r="D2" t="n">
-        <v>15445.2</v>
+        <v>16521.3</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -5383,7 +5807,6 @@
           <t>Segunda firma de la revision; EPP y candados LOTO van en la maleta personal, no en el carrito</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5445,7 +5868,6 @@
           <t>Asigna kits a frentes al publicar el plan; recibe escalaciones</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5463,7 +5885,6 @@
           <t>Responsable en EN_TRANSITO</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5545,7 +5966,6 @@
           <t>Base de un kit de taller o de un modulo en planta ancla</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5563,7 +5983,6 @@
           <t>Taller / camioneta</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5603,7 +6022,6 @@
           <t>Resguardo fijo en planta ancla cuando el cliente no da cuarto</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5643,7 +6061,6 @@
           <t>Van en su estuche con el modulo correspondiente</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5661,7 +6078,6 @@
           <t>Equipo mayor con su propio control</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5679,7 +6095,6 @@
           <t>Un juego por carrito; sobran 5 juegos Torx</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
herramientas-mx: juegos en huecos individuales y base 8410 + 8442 en lugar de la 8420 (#343, bloque 1)
Dadera con 29 dados parados y matraca aparte (medidas de Home Depot Mexico), regletas de un hueco por pieza para
desarmadores de precision, brocas, desarmadores Husky, adaptadores y extensiones. Brocas y adaptadores crecen con su
medida nominal. 8420 sustituida por 8410 + 8442 (opcion b). Interferencias 3D, estabilidad, costo, SVG, SCAD y STL del
C6 regenerados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TeXFoDoFpVre8AKoL589gf
</commit_message>
<xml_diff>
--- a/docs/herramientas-mx/asignacion_y_compra.xlsx
+++ b/docs/herramientas-mx/asignacion_y_compra.xlsx
@@ -16,7 +16,6 @@
     <sheet name="Fabricacion" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Asignacion_por_rol" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Reuso_inventario" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Cambios_sesion_nocturna" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39,7 +38,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -49,11 +48,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00B71C1C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001B5E20"/>
       </patternFill>
     </fill>
   </fills>
@@ -69,12 +63,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -488,7 +479,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>113195.3</v>
+        <v>116685.3</v>
       </c>
     </row>
     <row r="5">
@@ -518,7 +509,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>316214.8</v>
+        <v>319704.8</v>
       </c>
     </row>
     <row r="8">
@@ -528,7 +519,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>255551.74</v>
+        <v>259041.74</v>
       </c>
     </row>
     <row r="9">
@@ -538,7 +529,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>300352.37</v>
+        <v>303360.99</v>
       </c>
     </row>
     <row r="10">
@@ -548,7 +539,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>348408.75</v>
+        <v>351898.75</v>
       </c>
     </row>
     <row r="11">
@@ -570,339 +561,6 @@
       <c r="B12" t="inlineStr">
         <is>
           <t>17.64 MXN/USD (Odoo, 2026-09-27)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>concepto</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>antes (d8f4483)</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>ahora</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>diferencia</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Herramienta a comprar (conservador, solo renglones con precio)</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>159742.85</v>
-      </c>
-      <c r="C2" t="n">
-        <v>166422.1</v>
-      </c>
-      <c r="D2" t="n">
-        <v>6679.25</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Herramienta a comprar si aparecen las compras de Odoo posteriores al listado</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>99079.78999999999</v>
-      </c>
-      <c r="C3" t="n">
-        <v>105759.04</v>
-      </c>
-      <c r="D3" t="n">
-        <v>6679.25</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Contenedores, candados y cables</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>112491.3</v>
-      </c>
-      <c r="C4" t="n">
-        <v>113195.3</v>
-      </c>
-      <c r="D4" t="n">
-        <v>704</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>RFID (tags + lector)</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>20076.1</v>
-      </c>
-      <c r="C5" t="n">
-        <v>20076.1</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Filamento PETG</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>15445.2</v>
-      </c>
-      <c r="C6" t="n">
-        <v>16521.3</v>
-      </c>
-      <c r="D6" t="n">
-        <v>1076.1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>TOTAL con precio conocido (MXN, mezcla de precios sin IVA pagados y precios de tienda)</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>307755.45</v>
-      </c>
-      <c r="C7" t="n">
-        <v>316214.8</v>
-      </c>
-      <c r="D7" t="n">
-        <v>8459.35</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>TOTAL si aparecen las compras de Odoo</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>247092.39</v>
-      </c>
-      <c r="C8" t="n">
-        <v>255551.74</v>
-      </c>
-      <c r="D8" t="n">
-        <v>8459.35</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>TOTAL con precio conocido, normalizado SIN IVA (tienda / 1.16)</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>300352.37</v>
-      </c>
-      <c r="D9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>TOTAL normalizado con IVA (x 1.16)</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>348408.75</v>
-      </c>
-      <c r="D10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Renglones de herramienta SIN precio (cotizar)</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>9</v>
-      </c>
-      <c r="C11" t="n">
-        <v>5</v>
-      </c>
-      <c r="D11" t="n">
-        <v>-4</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Tipo de cambio usado</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>17.64 MXN/USD (Odoo, 2026-09-27)</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>17.64 MXN/USD (Odoo, 2026-09-27)</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>CONTENEDOR</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>necesidad antes</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>necesidad ahora</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>a comprar ahora</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>48-22-8420</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>6</v>
-      </c>
-      <c r="C15" t="n">
-        <v>6</v>
-      </c>
-      <c r="D15" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>48-22-8442</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>5</v>
-      </c>
-      <c r="C16" t="n">
-        <v>3</v>
-      </c>
-      <c r="D16" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>48-22-8443</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>2</v>
-      </c>
-      <c r="C17" t="n">
-        <v>7</v>
-      </c>
-      <c r="D17" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>48-22-8444</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>15</v>
-      </c>
-      <c r="C18" t="n">
-        <v>8</v>
-      </c>
-      <c r="D18" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>48-22-8447</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>4</v>
-      </c>
-      <c r="D19" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>POR QUE CAMBIO</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Mezcla de cajas del acomodo nuevo (base 8420 + 8443 + 8444 con M18 bajo candado; soldadura 2 x 8447); 5 renglones antes sin precio ya lo tienen (pagina Home Depot MX leida, IVA incluido); 8443 a $3,799 de la pagina HD MX (antes $3,399 de fragmento); PETG sube por mas cajones con pieza.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>IVA</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>La hoja Resumen trae ahora el total normalizado SIN IVA (precio de tienda / 1.16) y con IVA. Lo pagado en Odoo ya viene sin IVA.</t>
         </is>
       </c>
     </row>
@@ -964,7 +622,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1 x 48-22-8443 + 1 x 48-22-8444 + 1 x 48-22-8420</t>
+          <t>1 x 48-22-8443 + 1 x 48-22-8444 + 1 x 48-22-8442 + 1 x 48-22-8410</t>
         </is>
       </c>
     </row>
@@ -1135,10 +793,10 @@
         <v>24046.2</v>
       </c>
       <c r="D2" t="n">
-        <v>13369</v>
+        <v>14067</v>
       </c>
       <c r="E2" t="n">
-        <v>37415.2</v>
+        <v>38113.2</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4637,7 +4295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4759,158 +4417,190 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>48-22-8420</t>
+          <t>48-22-8442</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E4" t="n">
-        <v>5599</v>
+        <v>3952</v>
       </c>
       <c r="F4" t="n">
-        <v>33594</v>
+        <v>31616</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>buscador HerramientaElectrica.mx</t>
+          <t>buscador HerramientaElectrica.mx (agotado)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>alta</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>48-22-8447</t>
+          <t>48-22-8410</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E5" t="n">
-        <v>3499</v>
+        <v>2345</v>
       </c>
       <c r="F5" t="n">
-        <v>10497</v>
+        <v>11725</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Odoo P05566 (2026-02-04, sin IVA)</t>
+          <t>buscador Ferreterias Calzada, IVA incluido (leido 2026-09-28, #343)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>pagado</t>
+          <t>media</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>48-22-8442</t>
+          <t>48-22-8447</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
         <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>3952</v>
+        <v>3499</v>
       </c>
       <c r="F6" t="n">
-        <v>11856</v>
+        <v>10497</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>buscador HerramientaElectrica.mx (agotado)</t>
+          <t>Odoo P05566 (2026-02-04, sin IVA)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>pagado</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Candado de combinacion (1 por contenedor)</t>
+          <t>48-22-8420</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>119</v>
+        <v>5599</v>
       </c>
       <c r="F7" t="n">
-        <v>3332</v>
+        <v>5599</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>listado hoja Maleta Personal: Master 646DMX, Home Depot</t>
+          <t>buscador HerramientaElectrica.mx</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>pagado</t>
+          <t>media</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Candado de combinacion (1 por contenedor)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>28</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>28</v>
+      </c>
+      <c r="E8" t="n">
+        <v>119</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3332</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>listado hoja Maleta Personal: Master 646DMX, Home Depot</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>pagado</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Cable de acero con candado para resguardo (1 por kit + 1 por modulo con 8420)</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B9" t="n">
         <v>6</v>
       </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
         <v>6</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E9" t="n">
         <v>337.55</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F9" t="n">
         <v>2025.3</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>buscador Amazon MX: cable 1.8 m con combinacion reajustable</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>baja</t>
         </is>
@@ -5807,6 +5497,7 @@
           <t>Segunda firma de la revision; EPP y candados LOTO van en la maleta personal, no en el carrito</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5868,6 +5559,7 @@
           <t>Asigna kits a frentes al publicar el plan; recibe escalaciones</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5885,6 +5577,7 @@
           <t>Responsable en EN_TRANSITO</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5966,6 +5659,7 @@
           <t>Base de un kit de taller o de un modulo en planta ancla</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5983,6 +5677,7 @@
           <t>Taller / camioneta</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6022,6 +5717,7 @@
           <t>Resguardo fijo en planta ancla cuando el cliente no da cuarto</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6061,6 +5757,7 @@
           <t>Van en su estuche con el modulo correspondiente</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -6078,6 +5775,7 @@
           <t>Equipo mayor con su propio control</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6095,6 +5793,7 @@
           <t>Un juego por carrito; sobran 5 juegos Torx</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>